<commit_message>
Add AI stories to MO backlog
</commit_message>
<xml_diff>
--- a/product backlog template_v1_wxz.xlsx
+++ b/product backlog template_v1_wxz.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="29400" windowHeight="12540"/>
+    <workbookView windowWidth="24240" windowHeight="11480"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="80">
   <si>
     <t>Story ID</t>
   </si>
@@ -184,6 +184,66 @@
   <si>
     <t>1. For unfilled positions, the MO can modify its description, requirements, etc.
 2. The MO can manually set a job's status to "Closed".</t>
+  </si>
+  <si>
+    <t>Mo-009</t>
+  </si>
+  <si>
+    <t>Automatically extracts job position keywords</t>
+  </si>
+  <si>
+    <t>As a Module Organiser, I want the AI to automatically extract key skills/requirements from my job description, so that I don’t need to manually set screening criteria.</t>
+  </si>
+  <si>
+    <t>1.Given I paste a 200-500 word job description into the system.
+2. When I click "AI Extract Keywords", the system returns 5-8 core keywords 
+3. Then I can edit any keyword before confirming.
+4. If the description is less than 50 words, the system prompts "Please provide a more detailed description"</t>
+  </si>
+  <si>
+    <t>Mo-010</t>
+  </si>
+  <si>
+    <t>Generate Applicant Matching Report</t>
+  </si>
+  <si>
+    <t>As a Module Organiser, I want the AI to generate a candidate matching report, so that I can quickly understand an applicant’s suitability for the job.</t>
+  </si>
+  <si>
+    <t>1. Given I select an applicant for a specific job.
+2. When I click "View AI Match Report", the system shows a 0-100 score and a breakdown .
+3. The report highlights 3 key strengths  and 2 improvement areas.
+4. The report can be exported as a PDF file</t>
+  </si>
+  <si>
+    <t>Mo-011</t>
+  </si>
+  <si>
+    <t>Recommend similar applicants</t>
+  </si>
+  <si>
+    <t>As a Module Organiser, I want the AI to recommend candidates similar to the one I marked as "Preferred", so that I don’t miss potential suitable applicants.</t>
+  </si>
+  <si>
+    <t>1. Given I mark an applicant as "Preferred" on the applicant list.
+2. When I click "Find Similar Candidates", the system displays top 3 similar applicants within 5 seconds.
+3. The recommendation shows a "Similarity Score" (0-100) and the reason for recommendation .
+4. I can click "Dismiss" to remove an irrelevant recommendation.</t>
+  </si>
+  <si>
+    <t>Mo-012</t>
+  </si>
+  <si>
+    <t>Predict workload and generate scheduling suggestions</t>
+  </si>
+  <si>
+    <t>As a Module Organiser, I want the AI to predict the monthly workload of my hired TAs and generate a scheduling plan, so that I can avoid overloading or underutilizing TAs</t>
+  </si>
+  <si>
+    <t>1. Given I input the course details and the number of hired TAs.
+2. When I click "Generate Workload Plan", the AI calculates the monthly workload per TA  and breaks it down by task 
+3. The AI generates a weekly schedule table with no TA assigned more than 8 hours/week.
+4. I can adjust the schedule  and the AI automatically recalculates workload balance.</t>
   </si>
   <si>
     <t>ADM-001</t>
@@ -273,11 +333,9 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
+      <sz val="12"/>
       <name val="宋体"/>
       <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <u/>
@@ -742,19 +800,19 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -763,7 +821,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -885,7 +943,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -895,6 +953,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="27" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1244,7 +1314,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr defaultColWidth="8.83653846153846" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="1" width="11.5384615384615" style="1" customWidth="1"/>
@@ -1291,7 +1361,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" ht="118" spans="1:10">
+    <row r="2" ht="118" spans="3:6">
       <c r="C2" s="1" t="s">
         <v>10</v>
       </c>
@@ -1299,7 +1369,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" ht="84" spans="1:10">
+    <row r="3" ht="84" spans="1:6">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -1316,7 +1386,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" ht="84" spans="1:10">
+    <row r="4" ht="84" spans="1:6">
       <c r="A4" s="1" t="s">
         <v>16</v>
       </c>
@@ -1333,7 +1403,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" ht="51" spans="1:10">
+    <row r="5" ht="51" spans="1:6">
       <c r="A5" s="1" t="s">
         <v>20</v>
       </c>
@@ -1350,7 +1420,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" ht="101" spans="1:10">
+    <row r="6" ht="101" spans="1:6">
       <c r="A6" s="1" t="s">
         <v>24</v>
       </c>
@@ -1367,7 +1437,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" ht="68" spans="1:10">
+    <row r="7" ht="68" spans="1:6">
       <c r="A7" s="1" t="s">
         <v>28</v>
       </c>
@@ -1384,7 +1454,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" ht="118" spans="1:10">
+    <row r="8" ht="118" spans="1:6">
       <c r="A8" s="1" t="s">
         <v>32</v>
       </c>
@@ -1401,7 +1471,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="9" ht="118" spans="1:10">
+    <row r="9" ht="118" spans="1:6">
       <c r="A9" s="1" t="s">
         <v>36</v>
       </c>
@@ -1418,7 +1488,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="10" ht="101" spans="1:10">
+    <row r="10" ht="84" spans="1:6">
       <c r="A10" s="1" t="s">
         <v>40</v>
       </c>
@@ -1435,75 +1505,79 @@
         <v>43</v>
       </c>
     </row>
-    <row r="11" ht="51" spans="1:10">
+    <row r="11" ht="124" spans="1:6">
       <c r="A11" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="D11" s="1">
-        <v>1</v>
-      </c>
-      <c r="F11" s="1" t="s">
+      <c r="D11" s="6">
+        <v>2</v>
+      </c>
+      <c r="E11" s="6"/>
+      <c r="F11" s="7" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="12" ht="68" spans="1:10">
+    <row r="12" ht="106" spans="1:6">
       <c r="A12" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12" s="6">
         <v>2</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="E12" s="6"/>
+      <c r="F12" s="7" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="13" ht="68" spans="1:10">
+    <row r="13" ht="141" spans="1:6">
       <c r="A13" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C13" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="D13" s="1">
-        <v>2</v>
-      </c>
-      <c r="F13" s="1" t="s">
+      <c r="D13" s="6">
+        <v>3</v>
+      </c>
+      <c r="E13" s="6"/>
+      <c r="F13" s="7" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="14" ht="84" spans="1:10">
+    <row r="14" ht="141" spans="1:6">
       <c r="A14" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="D14" s="1">
-        <v>3</v>
-      </c>
-      <c r="F14" s="1" t="s">
+      <c r="D14" s="6">
+        <v>2</v>
+      </c>
+      <c r="E14" s="6"/>
+      <c r="F14" s="7" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="15" ht="84" spans="1:10">
+    <row r="15" ht="51" spans="1:6">
       <c r="A15" s="1" t="s">
         <v>60</v>
       </c>
@@ -1514,10 +1588,78 @@
         <v>62</v>
       </c>
       <c r="D15" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>63</v>
+      </c>
+    </row>
+    <row r="16" ht="68" spans="1:6">
+      <c r="A16" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D16" s="1">
+        <v>2</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="17" ht="68" spans="1:6">
+      <c r="A17" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D17" s="1">
+        <v>2</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="18" ht="84" spans="1:6">
+      <c r="A18" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D18" s="1">
+        <v>3</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="19" ht="84" spans="1:6">
+      <c r="A19" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="D19" s="1">
+        <v>4</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add AI story to Admin backlog
</commit_message>
<xml_diff>
--- a/product backlog template_v1_wxz.xlsx
+++ b/product backlog template_v1_wxz.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="24240" windowHeight="11480"/>
+    <workbookView windowWidth="26760" windowHeight="11480"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="84">
   <si>
     <t>Story ID</t>
   </si>
@@ -148,7 +148,7 @@
     <t>Filter applications(AI function)</t>
   </si>
   <si>
-    <t>As an MO, I want the system to automatically filter and rank applicants based on the job's required skills, so that I can quickly identify the most suitable candidates.</t>
+    <t>As a Module Organiser I want the system to automatically filter and rank applicants based on the job's required skills, so that I can quickly identify the most suitable candidates.</t>
   </si>
   <si>
     <t>1. On the applicant list page, there is an "Sort" or "Smart Rank" button.
@@ -312,6 +312,21 @@
   <si>
     <t>1. When an MO attempts to hire a TA who is already holding multiple positions, the system displays a warning: "This TA already holds X positions. Consider other candidates."
 2. The system can suggest alternative, equally qualified candidates with a lighter workload.</t>
+  </si>
+  <si>
+    <t>ADM-006</t>
+  </si>
+  <si>
+    <t>Generate recruitment data report</t>
+  </si>
+  <si>
+    <t>As a System Admin, I want the AI to generate monthly recruitment data reports, so that I can analyze the system’s usage efficiency.</t>
+  </si>
+  <si>
+    <t>1. Given it’s the 1st day of the month.
+2. The AI automatically generates a report with 5 sections: "Job Post Volume", "Application Volume", "AI Match Score Distribution", "Hiring Rate", "MO Satisfaction Score".
+3. The report includes visual charts (line charts, pie charts) and 3 key insights .
+4. The report can be shared with MOs via email.</t>
   </si>
 </sst>
 </file>
@@ -1314,7 +1329,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:J20"/>
   <sheetFormatPr defaultColWidth="8.83653846153846" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="1" width="11.5384615384615" style="1" customWidth="1"/>
@@ -1662,6 +1677,24 @@
         <v>79</v>
       </c>
     </row>
+    <row r="20" ht="124" spans="1:6">
+      <c r="A20" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="D20" s="6">
+        <v>3</v>
+      </c>
+      <c r="E20" s="6"/>
+      <c r="F20" s="7" t="s">
+        <v>83</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200"/>

</xml_diff>